<commit_message>
Add multi-stock forecast - 5 companies compared over 30 days
</commit_message>
<xml_diff>
--- a/project_details.xlsx
+++ b/project_details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ML-Projects\stocksense\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4901C05F-C937-4A22-89CA-C9E2E61DD4C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7324E7-8F2F-4B7F-BC24-9ABDD7C4B48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="98">
   <si>
     <t>But first — a concept to understand:</t>
   </si>
@@ -591,6 +591,90 @@
       </rPr>
       <t>"</t>
     </r>
+  </si>
+  <si>
+    <t>Now let's take stock of what StockSense has so far:</t>
+  </si>
+  <si>
+    <t>stocksense/</t>
+  </si>
+  <si>
+    <t>├── 01_explore_stocks.py      ✅ data exploration + chart</t>
+  </si>
+  <si>
+    <t>├── 02_prepare_data.py        ✅ data prep for Prophet</t>
+  </si>
+  <si>
+    <t>├── 03_train_prophet.py       ✅ model training + evaluation</t>
+  </si>
+  <si>
+    <t>├── 04_forecast_future.py     ✅ 30-day future forecast</t>
+  </si>
+  <si>
+    <t>├── 05_components.py          ✅ trend/seasonality breakdown</t>
+  </si>
+  <si>
+    <t>├── data/</t>
+  </si>
+  <si>
+    <t>│   └── apple_prophet.csv     ✅ prepared dataset</t>
+  </si>
+  <si>
+    <t>├── apple_price_history.png   ✅ historical price chart</t>
+  </si>
+  <si>
+    <t>├── forecast_vs_actual.png    ✅ forecast accuracy chart</t>
+  </si>
+  <si>
+    <t>├── future_forecast.png       ✅ 30-day forecast chart</t>
+  </si>
+  <si>
+    <t>├── forecast_components.png   ✅ component breakdown</t>
+  </si>
+  <si>
+    <t>└── changepoints.png          ✅ trend change points</t>
+  </si>
+  <si>
+    <r>
+      <t>This is called "competing signals" in forecasting</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — when trend and seasonality pull in opposite directions, the model has to balance both. The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>changepoint_prior_scale=0.05</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> parameter we set controls this balance — a lower value makes the trend more conservative, a higher value makes it follow recent momentum more aggressively.</t>
+    </r>
+  </si>
+  <si>
+    <t>In your interview you could say:</t>
+  </si>
+  <si>
+    <t>"I noticed a conflict between Apple's negative June-July yearly seasonality and its strong 2026 upward trend. Prophet balanced both signals, producing a moderate bullish forecast. If I were deploying this in production, I would monitor whether the seasonal pattern or the momentum dominates — and potentially adjust the changepoint_prior_scale parameter to reflect current market conditions."</t>
+  </si>
+  <si>
+    <t>That is Principal-level thinking — not just running a model but understanding and questioning its assumptions.</t>
   </si>
 </sst>
 </file>
@@ -697,7 +781,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -735,6 +819,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1128,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4F31BBB-9CF1-491D-877F-7E4AA6629DFA}">
-  <dimension ref="A2:D146"/>
+  <dimension ref="A2:D173"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="81.77734375" style="2" customWidth="1"/>
@@ -1324,57 +1414,61 @@
         <v>46</v>
       </c>
     </row>
-    <row r="97" spans="2:2">
+    <row r="97" spans="1:2">
       <c r="B97" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="99" spans="2:2" ht="28.8">
+    <row r="99" spans="1:2" ht="28.8">
       <c r="B99" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="101" spans="2:2" ht="57.6">
+    <row r="101" spans="1:2" ht="57.6">
       <c r="B101" s="10" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="103" spans="2:2">
+    <row r="103" spans="1:2">
       <c r="B103" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="105" spans="2:2">
+    <row r="104" spans="1:2">
+      <c r="A104" s="5"/>
+      <c r="B104" s="6"/>
+    </row>
+    <row r="105" spans="1:2">
       <c r="B105" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="106" spans="2:2">
+    <row r="106" spans="1:2">
       <c r="B106" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="1:2">
       <c r="B107" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="108" spans="2:2">
+    <row r="108" spans="1:2">
       <c r="B108" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="109" spans="2:2">
+    <row r="109" spans="1:2">
       <c r="B109" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="110" spans="2:2">
+    <row r="110" spans="1:2">
       <c r="B110" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="112" spans="2:2">
+    <row r="112" spans="1:2">
       <c r="B112" s="2" t="s">
         <v>56</v>
       </c>
@@ -1561,19 +1655,121 @@
       <c r="C144" s="2"/>
       <c r="D144" s="2"/>
     </row>
-    <row r="145" spans="2:4">
+    <row r="145" spans="1:4">
       <c r="C145" s="2"/>
       <c r="D145" s="2"/>
     </row>
-    <row r="146" spans="2:4" ht="57.6">
+    <row r="146" spans="1:4" ht="57.6">
       <c r="B146" s="10" t="s">
         <v>79</v>
       </c>
       <c r="C146" s="2"/>
       <c r="D146" s="2"/>
     </row>
+    <row r="148" spans="1:4">
+      <c r="A148" s="5"/>
+      <c r="B148" s="6"/>
+    </row>
+    <row r="149" spans="1:4">
+      <c r="B149" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4">
+      <c r="B150"/>
+    </row>
+    <row r="151" spans="1:4">
+      <c r="B151" s="14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4">
+      <c r="B152" s="14" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4">
+      <c r="B153" s="14" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4">
+      <c r="B154" s="14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4">
+      <c r="B155" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4">
+      <c r="B156" s="14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4">
+      <c r="B157" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4">
+      <c r="B158" s="14" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4">
+      <c r="B159" s="14" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4">
+      <c r="B160" s="14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="B161" s="14" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="B162" s="14" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="B163" s="14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="5"/>
+      <c r="B165" s="6"/>
+    </row>
+    <row r="167" spans="1:2" ht="57.6">
+      <c r="B167" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="B169" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" ht="72">
+      <c r="B171" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" ht="28.8">
+      <c r="B173" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add MLflow tracking and forecast chatbot - StockSense complete
</commit_message>
<xml_diff>
--- a/project_details.xlsx
+++ b/project_details.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ML-Projects\stocksense\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7324E7-8F2F-4B7F-BC24-9ABDD7C4B48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C4B48BB-EFF2-4A23-88BB-16F0E29190FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="126">
   <si>
     <t>But first — a concept to understand:</t>
   </si>
@@ -675,6 +676,150 @@
   </si>
   <si>
     <t>That is Principal-level thinking — not just running a model but understanding and questioning its assumptions.</t>
+  </si>
+  <si>
+    <t>Let's look at what you've built across both projects:</t>
+  </si>
+  <si>
+    <r>
+      <t>Project 1 — FinSight AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ✅</t>
+    </r>
+  </si>
+  <si>
+    <t>Data engineering + ML + MLOps + RAG chatbot + Airflow orchestration</t>
+  </si>
+  <si>
+    <r>
+      <t>Project 2 — StockSense</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ✅</t>
+    </r>
+  </si>
+  <si>
+    <t>Time series forecasting + component analysis + multi-stock comparison</t>
+  </si>
+  <si>
+    <t>What StockSense added to your portfolio that FinSight AI didn't have:</t>
+  </si>
+  <si>
+    <t>A completely different ML problem type (forecasting vs classification)</t>
+  </si>
+  <si>
+    <t>Time series concepts (seasonality, trend, changepoints)</t>
+  </si>
+  <si>
+    <t>Prophet decomposition and component analysis</t>
+  </si>
+  <si>
+    <t>MAPE/MAE/RMSE evaluation metrics</t>
+  </si>
+  <si>
+    <t>Critical thinking about model limitations</t>
+  </si>
+  <si>
+    <t>Your portfolio now covers:</t>
+  </si>
+  <si>
+    <t>Skill</t>
+  </si>
+  <si>
+    <t>Project</t>
+  </si>
+  <si>
+    <t>Data ingestion &amp; warehousing</t>
+  </si>
+  <si>
+    <t>FinSight AI</t>
+  </si>
+  <si>
+    <t>Classification ML</t>
+  </si>
+  <si>
+    <t>MLOps &amp; model registry</t>
+  </si>
+  <si>
+    <t>RAG &amp; GenAI</t>
+  </si>
+  <si>
+    <t>Airflow orchestration</t>
+  </si>
+  <si>
+    <t>Time series forecasting</t>
+  </si>
+  <si>
+    <t>StockSense</t>
+  </si>
+  <si>
+    <t>Seasonality analysis</t>
+  </si>
+  <si>
+    <t>Multi-model comparison</t>
+  </si>
+  <si>
+    <t>Remaining projects:</t>
+  </si>
+  <si>
+    <r>
+      <t>Project 3 — NewsRisk</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (NLP sentiment analysis on financial news)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Project 4 — StreamAlert</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (real-time fraud detection with Kafka)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Project 5 — AzureFinSight</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (deploy FinSight AI on Azure)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -781,7 +926,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -823,8 +968,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1758,7 +1913,7 @@
       </c>
     </row>
     <row r="171" spans="1:2" ht="72">
-      <c r="B171" s="15" t="s">
+      <c r="B171" s="16" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1772,4 +1927,176 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{989866FA-49AE-4742-B55B-0979CDD02F2B}">
+  <dimension ref="B2:C39"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="60.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2">
+      <c r="B4" s="15" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2">
+      <c r="B5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2">
+      <c r="B7" s="15" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2">
+      <c r="B8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2">
+      <c r="B12" s="15" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2">
+      <c r="B13" s="17"/>
+    </row>
+    <row r="14" spans="2:2">
+      <c r="B14" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2">
+      <c r="B15" s="17" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2">
+      <c r="B16" s="17" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="17" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3">
+      <c r="B22" s="15" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3">
+      <c r="B24" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3">
+      <c r="B25" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3">
+      <c r="B26" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3">
+      <c r="B27" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3">
+      <c r="B28" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3">
+      <c r="B29" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3">
+      <c r="B30" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3">
+      <c r="B31" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3">
+      <c r="B32" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36" s="17"/>
+    </row>
+    <row r="37" spans="2:2">
+      <c r="B37" s="18" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2">
+      <c r="B38" s="18" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2">
+      <c r="B39" s="18" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
- StockSense project project details txt,xlsx changes done
</commit_message>
<xml_diff>
--- a/project_details.xlsx
+++ b/project_details.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ML-Projects\stocksense\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C4B48BB-EFF2-4A23-88BB-16F0E29190FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80FA7FBB-1183-430B-892C-6A0C325F74A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="157">
   <si>
     <t>But first — a concept to understand:</t>
   </si>
@@ -820,6 +821,122 @@
       </rPr>
       <t xml:space="preserve"> (deploy FinSight AI on Azure)</t>
     </r>
+  </si>
+  <si>
+    <t>Final StockSense file structure:</t>
+  </si>
+  <si>
+    <t>├── 01_explore_stocks.py       ✅ data exploration</t>
+  </si>
+  <si>
+    <t>├── 02_prepare_data.py         ✅ Prophet data preparation</t>
+  </si>
+  <si>
+    <t>├── 03_train_prophet.py        ✅ model training + evaluation</t>
+  </si>
+  <si>
+    <t>├── 04_forecast_future.py      ✅ 30-day future forecast</t>
+  </si>
+  <si>
+    <t>├── 05_components.py           ✅ trend/seasonality breakdown</t>
+  </si>
+  <si>
+    <t>├── 06_multi_stock_forecast.py ✅ 5-company comparison</t>
+  </si>
+  <si>
+    <t>├── 07_mlflow_tracking.py      ✅ MLflow experiment tracking</t>
+  </si>
+  <si>
+    <t>├── 08_forecast_chatbot.py     ✅ Phi-3 forecast chatbot</t>
+  </si>
+  <si>
+    <t>└── README.md                  ✅ documentation</t>
+  </si>
+  <si>
+    <t>What StockSense added to your portfolio:</t>
+  </si>
+  <si>
+    <t>Demonstrated</t>
+  </si>
+  <si>
+    <t>Prophet on real stock data</t>
+  </si>
+  <si>
+    <t>Weekly + yearly patterns identified</t>
+  </si>
+  <si>
+    <t>5 stocks tracked simultaneously</t>
+  </si>
+  <si>
+    <t>MLflow for forecasting</t>
+  </si>
+  <si>
+    <t>MAPE comparison across stocks</t>
+  </si>
+  <si>
+    <t>Architectural judgment</t>
+  </si>
+  <si>
+    <t>Simple injection vs full RAG decision</t>
+  </si>
+  <si>
+    <t>Critical model evaluation</t>
+  </si>
+  <si>
+    <t>Honest assessment of Prophet's limitations</t>
+  </si>
+  <si>
+    <t>Portfolio status so far:</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>✅ Complete</t>
+  </si>
+  <si>
+    <t>NewsRisk</t>
+  </si>
+  <si>
+    <t>⏳ Next</t>
+  </si>
+  <si>
+    <t>StreamAlert</t>
+  </si>
+  <si>
+    <t>⏳ Pending</t>
+  </si>
+  <si>
+    <t>AzureFinSight</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">When you are ready say </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"ready to start NewsRisk"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and we begin Project 3 — NLP sentiment analysis on financial news.</t>
+    </r>
+  </si>
+  <si>
+    <t>You are making excellent progress.</t>
   </si>
 </sst>
 </file>
@@ -2099,4 +2216,201 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78CBDEB7-2876-4CD4-B3C6-090A9A355D9F}">
+  <dimension ref="B2:C40"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="69.109375" customWidth="1"/>
+    <col min="3" max="3" width="50.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2">
+      <c r="B4" s="14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2">
+      <c r="B5" s="14" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2">
+      <c r="B6" s="14" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2">
+      <c r="B7" s="14" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2">
+      <c r="B8" s="14" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2">
+      <c r="B9" s="14" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2">
+      <c r="B10" s="14" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2">
+      <c r="B11" s="14" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2">
+      <c r="B12" s="14" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2">
+      <c r="B13" s="14" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="B20" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3">
+      <c r="B21" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3">
+      <c r="B22" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3">
+      <c r="B23" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3">
+      <c r="B24" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3">
+      <c r="B25" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3">
+      <c r="B28" s="15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3">
+      <c r="B30" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3">
+      <c r="B31" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3">
+      <c r="B32" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3">
+      <c r="B33" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3">
+      <c r="B34" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="C34" s="19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3">
+      <c r="B35" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" s="19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3">
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+    </row>
+    <row r="38" spans="2:3">
+      <c r="B38" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3">
+      <c r="B40" t="s">
+        <v>156</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>